<commit_message>
Spreadsheet now displays better colors for Match errors.
</commit_message>
<xml_diff>
--- a/The Blue Alliance/Game Years/2026/2026nyro/tba_push_into_excel_template.xlsx
+++ b/The Blue Alliance/Game Years/2026/2026nyro/tba_push_into_excel_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/johnhurrell/Development/fairport-robotics/ScoutingPASSSync/tba/data/2026/2026nyro/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/johnhurrell/Development/fairport-robotics/ScoutingPASSSync/The Blue Alliance/Game Years/2026/2026nyro/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{789C64D7-C901-8345-BDA2-6E91BB216C0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B82B372-5382-7A4A-96E4-798DCC37501E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MatchScoutingData" sheetId="1" r:id="rId1"/>
@@ -71,7 +71,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2114" uniqueCount="610">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2118" uniqueCount="614">
   <si>
     <t>Key</t>
   </si>
@@ -1902,6 +1902,18 @@
   <si>
     <t>83.Red 3</t>
   </si>
+  <si>
+    <t>Match has not yet been scouted</t>
+  </si>
+  <si>
+    <t>Match has been scouted</t>
+  </si>
+  <si>
+    <t>Match was scouted more than once</t>
+  </si>
+  <si>
+    <t>Wrong team was scouted</t>
+  </si>
 </sst>
 </file>
 
@@ -1910,7 +1922,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0;\-0;;@"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1970,8 +1982,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2023,6 +2042,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC8D6A1"/>
+        <bgColor rgb="FFC8D6A1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2117,7 +2148,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2138,33 +2169,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
@@ -2195,6 +2199,38 @@
     <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2518,91 +2554,91 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:29" ht="125" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="21" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="21" t="s">
+      <c r="A1" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="C1" s="21" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="21" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="21" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="21" t="s">
+      <c r="C1" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="G1" s="21" t="s">
+      <c r="G1" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="H1" s="21" t="s">
+      <c r="H1" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="I1" s="21" t="s">
+      <c r="I1" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="J1" s="21" t="s">
+      <c r="J1" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="K1" s="21" t="s">
+      <c r="K1" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="L1" s="21" t="s">
+      <c r="L1" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="M1" s="21" t="s">
+      <c r="M1" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="N1" s="21" t="s">
+      <c r="N1" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="O1" s="21" t="s">
+      <c r="O1" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="P1" s="21" t="s">
+      <c r="P1" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="Q1" s="21" t="s">
+      <c r="Q1" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="R1" s="21" t="s">
+      <c r="R1" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="S1" s="21" t="s">
+      <c r="S1" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="T1" s="21" t="s">
+      <c r="T1" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="U1" s="21" t="s">
+      <c r="U1" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="V1" s="21" t="s">
+      <c r="V1" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="W1" s="21" t="s">
+      <c r="W1" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="X1" s="21" t="s">
+      <c r="X1" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="Y1" s="21" t="s">
+      <c r="Y1" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="Z1" s="21" t="s">
+      <c r="Z1" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="AA1" s="21" t="s">
+      <c r="AA1" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="AB1" s="21" t="s">
+      <c r="AB1" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="AC1" s="21" t="s">
+      <c r="AC1" s="12" t="s">
         <v>4</v>
       </c>
     </row>
@@ -56994,7 +57030,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -57003,7 +57039,7 @@
     <col min="10" max="10" width="35.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
         <v>1</v>
       </c>
@@ -57028,6 +57064,56 @@
       <c r="H1" s="10" t="s">
         <v>81</v>
       </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J2" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J3" s="31" t="s">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J4" s="35" t="s">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J5" s="32" t="s">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J6" s="32"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J7" s="33"/>
+    </row>
+    <row r="8" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+      <c r="J8" s="34"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J9" s="33"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J10" s="33"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J11" s="33"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J12" s="33"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J13" s="33"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J14" s="33"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J15" s="33"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:H1" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
@@ -57078,116 +57164,116 @@
     <row r="1" spans="1:26" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6"/>
       <c r="B1" s="6"/>
-      <c r="C1" s="14" t="s">
+      <c r="C1" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="15"/>
-      <c r="H1" s="16" t="s">
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
-      <c r="K1" s="17"/>
-      <c r="L1" s="17"/>
-      <c r="M1" s="17"/>
-      <c r="N1" s="17"/>
-      <c r="O1" s="17"/>
-      <c r="P1" s="18" t="s">
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
+      <c r="K1" s="27"/>
+      <c r="L1" s="27"/>
+      <c r="M1" s="27"/>
+      <c r="N1" s="27"/>
+      <c r="O1" s="27"/>
+      <c r="P1" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="Q1" s="19"/>
-      <c r="R1" s="19"/>
-      <c r="S1" s="19"/>
-      <c r="T1" s="19"/>
-      <c r="U1" s="12" t="s">
+      <c r="Q1" s="29"/>
+      <c r="R1" s="29"/>
+      <c r="S1" s="29"/>
+      <c r="T1" s="29"/>
+      <c r="U1" s="22" t="s">
         <v>72</v>
       </c>
-      <c r="V1" s="12"/>
-      <c r="W1" s="12"/>
-      <c r="X1" s="12"/>
-      <c r="Y1" s="12"/>
-      <c r="Z1" s="13"/>
+      <c r="V1" s="22"/>
+      <c r="W1" s="22"/>
+      <c r="X1" s="22"/>
+      <c r="Y1" s="22"/>
+      <c r="Z1" s="23"/>
     </row>
     <row r="2" spans="1:26" ht="130" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="23" t="s">
+      <c r="A2" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="C2" s="24" t="s">
+      <c r="C2" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="D2" s="24" t="s">
+      <c r="D2" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="E2" s="24" t="s">
+      <c r="E2" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="F2" s="24" t="s">
+      <c r="F2" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="G2" s="24" t="s">
+      <c r="G2" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="H2" s="25" t="s">
+      <c r="H2" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="I2" s="25" t="s">
+      <c r="I2" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="J2" s="25" t="s">
+      <c r="J2" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="K2" s="25" t="s">
+      <c r="K2" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="L2" s="25" t="s">
+      <c r="L2" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="M2" s="25" t="s">
+      <c r="M2" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="N2" s="25" t="s">
+      <c r="N2" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="O2" s="25" t="s">
+      <c r="O2" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="P2" s="26" t="s">
+      <c r="P2" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="Q2" s="26" t="s">
+      <c r="Q2" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="R2" s="26" t="s">
+      <c r="R2" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="S2" s="26" t="s">
+      <c r="S2" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="T2" s="26" t="s">
+      <c r="T2" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="U2" s="27" t="s">
+      <c r="U2" s="18" t="s">
         <v>73</v>
       </c>
-      <c r="V2" s="27" t="s">
+      <c r="V2" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="W2" s="27" t="s">
+      <c r="W2" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="X2" s="27" t="s">
+      <c r="X2" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="Y2" s="27" t="s">
+      <c r="Y2" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="Z2" s="28" t="s">
+      <c r="Z2" s="19" t="s">
         <v>71</v>
       </c>
     </row>
@@ -65530,138 +65616,138 @@
     <row r="1" spans="1:31" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6"/>
       <c r="B1" s="6"/>
-      <c r="C1" s="14" t="s">
+      <c r="C1" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="15"/>
-      <c r="H1" s="16" t="s">
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
-      <c r="K1" s="17"/>
-      <c r="L1" s="17"/>
-      <c r="M1" s="17"/>
-      <c r="N1" s="17"/>
-      <c r="O1" s="17"/>
-      <c r="P1" s="18" t="s">
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
+      <c r="K1" s="27"/>
+      <c r="L1" s="27"/>
+      <c r="M1" s="27"/>
+      <c r="N1" s="27"/>
+      <c r="O1" s="27"/>
+      <c r="P1" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="Q1" s="19"/>
-      <c r="R1" s="19"/>
-      <c r="S1" s="19"/>
-      <c r="T1" s="19"/>
-      <c r="U1" s="12" t="s">
+      <c r="Q1" s="29"/>
+      <c r="R1" s="29"/>
+      <c r="S1" s="29"/>
+      <c r="T1" s="29"/>
+      <c r="U1" s="22" t="s">
         <v>72</v>
       </c>
-      <c r="V1" s="12"/>
-      <c r="W1" s="12"/>
-      <c r="X1" s="12"/>
-      <c r="Y1" s="12"/>
-      <c r="Z1" s="12"/>
-      <c r="AA1" s="20" t="s">
+      <c r="V1" s="22"/>
+      <c r="W1" s="22"/>
+      <c r="X1" s="22"/>
+      <c r="Y1" s="22"/>
+      <c r="Z1" s="22"/>
+      <c r="AA1" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="AB1" s="20"/>
-      <c r="AC1" s="20"/>
-      <c r="AD1" s="20"/>
-      <c r="AE1" s="20"/>
+      <c r="AB1" s="30"/>
+      <c r="AC1" s="30"/>
+      <c r="AD1" s="30"/>
+      <c r="AE1" s="30"/>
     </row>
     <row r="2" spans="1:31" ht="130" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="23" t="s">
+      <c r="A2" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="C2" s="24" t="s">
+      <c r="C2" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="D2" s="24" t="s">
+      <c r="D2" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="E2" s="24" t="s">
+      <c r="E2" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="F2" s="24" t="s">
+      <c r="F2" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="G2" s="24" t="s">
+      <c r="G2" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="H2" s="25" t="s">
+      <c r="H2" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="I2" s="25" t="s">
+      <c r="I2" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="J2" s="25" t="s">
+      <c r="J2" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="K2" s="25" t="s">
+      <c r="K2" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="L2" s="25" t="s">
+      <c r="L2" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="M2" s="25" t="s">
+      <c r="M2" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="N2" s="25" t="s">
+      <c r="N2" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="O2" s="25" t="s">
+      <c r="O2" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="P2" s="26" t="s">
+      <c r="P2" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="Q2" s="26" t="s">
+      <c r="Q2" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="R2" s="26" t="s">
+      <c r="R2" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="S2" s="26" t="s">
+      <c r="S2" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="T2" s="26" t="s">
+      <c r="T2" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="U2" s="27" t="s">
+      <c r="U2" s="18" t="s">
         <v>73</v>
       </c>
-      <c r="V2" s="27" t="s">
+      <c r="V2" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="W2" s="27" t="s">
+      <c r="W2" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="X2" s="27" t="s">
+      <c r="X2" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="Y2" s="27" t="s">
+      <c r="Y2" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="Z2" s="28" t="s">
+      <c r="Z2" s="19" t="s">
         <v>71</v>
       </c>
-      <c r="AA2" s="24" t="s">
+      <c r="AA2" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="AB2" s="25" t="s">
+      <c r="AB2" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="AC2" s="26" t="s">
+      <c r="AC2" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="AD2" s="29" t="s">
+      <c r="AD2" s="20" t="s">
         <v>72</v>
       </c>
-      <c r="AE2" s="30" t="s">
+      <c r="AE2" s="21" t="s">
         <v>75</v>
       </c>
     </row>

</xml_diff>